<commit_message>
integrated new google news library
</commit_message>
<xml_diff>
--- a/output/combined_output_adjusted.xlsx
+++ b/output/combined_output_adjusted.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/projects/rip-current/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23025917-BEE7-C34C-BEE3-2DA866541309}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{408AD6A7-7C14-BA45-A5EB-C8359D63CD67}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38180" yWindow="-640" windowWidth="35680" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37980" yWindow="-1020" windowWidth="35680" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="combined_output" sheetId="1" r:id="rId1"/>

</xml_diff>